<commit_message>
Update COMI and GOUR valuation models
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Gourmet-Egypt-GOUR-Valuation-Model.xlsx
+++ b/models/Gourmet-Egypt-GOUR-Valuation-Model.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahmed Wael\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC04101-24BD-4361-AE5C-F94309F1C380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62938B30-2935-4CAA-A52E-E014B389B9FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="646" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3732,16 +3732,16 @@
     <v>4</v>
     <v>54.81</v>
     <v>46.6</v>
-    <v>-0.01</v>
-    <v>-1.9130000000000001E-4</v>
+    <v>-0.03</v>
+    <v>-5.731E-4</v>
     <v>EGP</v>
     <v>USD</v>
     <v>Currency Pair</v>
-    <v>46298.209421296298</v>
+    <v>46304.208275462966</v>
     <v>US Dollar/Egyptian Pound FX Spot Rate</v>
-    <v>52.26</v>
-    <v>52.27</v>
-    <v>52.26</v>
+    <v>52.32</v>
+    <v>52.35</v>
+    <v>52.32</v>
     <v>USDEGP</v>
     <v>USD/EGP</v>
   </rv>
@@ -3893,7 +3893,7 @@
       <x:numFmt numFmtId="0" formatCode="General"/>
     </x:dxf>
     <x:dxf>
-      <x:numFmt numFmtId="27" formatCode="dd/mm/yy\ h:mm"/>
+      <x:numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
     </x:dxf>
     <x:dxf>
       <x:numFmt numFmtId="14" formatCode="0.00%"/>
@@ -8526,35 +8526,35 @@
         <v>29</v>
       </c>
       <c r="D173" s="36">
-        <f>D172/D16</f>
+        <f t="shared" ref="D173:K173" si="123">D172/D16</f>
         <v>2.5811960598944833E-2</v>
       </c>
       <c r="E173" s="36">
-        <f>E172/E16</f>
+        <f t="shared" si="123"/>
         <v>2.037199496176352E-2</v>
       </c>
       <c r="F173" s="36">
-        <f>F172/F16</f>
+        <f t="shared" si="123"/>
         <v>1.5037648838504851E-2</v>
       </c>
       <c r="G173" s="36">
-        <f>G172/G16</f>
+        <f t="shared" si="123"/>
         <v>1.4619590793516437E-2</v>
       </c>
       <c r="H173" s="36">
-        <f>H172/H16</f>
+        <f t="shared" si="123"/>
         <v>1.383263899959546E-2</v>
       </c>
       <c r="I173" s="36">
-        <f>I172/I16</f>
+        <f t="shared" si="123"/>
         <v>1.3465393048320895E-2</v>
       </c>
       <c r="J173" s="36">
-        <f>J172/J16</f>
+        <f t="shared" si="123"/>
         <v>1.3188195048879053E-2</v>
       </c>
       <c r="K173" s="36">
-        <f>K172/K16</f>
+        <f t="shared" si="123"/>
         <v>1.2966907635529074E-2</v>
       </c>
     </row>
@@ -8567,31 +8567,31 @@
         <v>82799438</v>
       </c>
       <c r="E174" s="30">
-        <f t="shared" ref="E174:K174" si="123">E164+E172</f>
+        <f t="shared" ref="E174:K174" si="124">E164+E172</f>
         <v>86351074</v>
       </c>
       <c r="F174" s="30">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>84629058</v>
       </c>
       <c r="G174" s="30">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>86759301.032923192</v>
       </c>
       <c r="H174" s="30">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>92694527.222767293</v>
       </c>
       <c r="I174" s="30">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>109883130.65339704</v>
       </c>
       <c r="J174" s="30">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>126905436.19804949</v>
       </c>
       <c r="K174" s="30">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>143591405.04245025</v>
       </c>
     </row>
@@ -8613,35 +8613,35 @@
         <v>107</v>
       </c>
       <c r="D177" s="48">
-        <f t="shared" ref="D177:K177" si="124">D$13</f>
+        <f t="shared" ref="D177:K177" si="125">D$13</f>
         <v>2023</v>
       </c>
       <c r="E177" s="48">
-        <f t="shared" si="124"/>
+        <f t="shared" si="125"/>
         <v>2024</v>
       </c>
       <c r="F177" s="48">
-        <f t="shared" si="124"/>
+        <f t="shared" si="125"/>
         <v>2025</v>
       </c>
       <c r="G177" s="49">
-        <f t="shared" si="124"/>
+        <f t="shared" si="125"/>
         <v>2026</v>
       </c>
       <c r="H177" s="49">
-        <f t="shared" si="124"/>
+        <f t="shared" si="125"/>
         <v>2027</v>
       </c>
       <c r="I177" s="49">
-        <f t="shared" si="124"/>
+        <f t="shared" si="125"/>
         <v>2028</v>
       </c>
       <c r="J177" s="49">
-        <f t="shared" si="124"/>
+        <f t="shared" si="125"/>
         <v>2029</v>
       </c>
       <c r="K177" s="49">
-        <f t="shared" si="124"/>
+        <f t="shared" si="125"/>
         <v>2030</v>
       </c>
     </row>
@@ -8650,35 +8650,35 @@
         <v>108</v>
       </c>
       <c r="D178" s="43">
-        <f t="shared" ref="D178:K178" si="125">D$14</f>
+        <f t="shared" ref="D178:K178" si="126">D$14</f>
         <v>45291</v>
       </c>
       <c r="E178" s="43">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>45657</v>
       </c>
       <c r="F178" s="43">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>46022</v>
       </c>
       <c r="G178" s="43">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>46387</v>
       </c>
       <c r="H178" s="43">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>46752</v>
       </c>
       <c r="I178" s="43">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>47118</v>
       </c>
       <c r="J178" s="43">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>47483</v>
       </c>
       <c r="K178" s="43">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>47848</v>
       </c>
     </row>
@@ -8708,19 +8708,19 @@
         <v>3519895922.2399998</v>
       </c>
       <c r="H180" s="330">
-        <f t="shared" ref="H180:K180" si="126">G180*(1+H189)</f>
+        <f t="shared" ref="H180:K180" si="127">G180*(1+H189)</f>
         <v>4153477188.2431993</v>
       </c>
       <c r="I180" s="330">
-        <f t="shared" si="126"/>
+        <f t="shared" si="127"/>
         <v>4776498766.4796791</v>
       </c>
       <c r="J180" s="330">
-        <f t="shared" si="126"/>
+        <f t="shared" si="127"/>
         <v>5349678618.4572411</v>
       </c>
       <c r="K180" s="330">
-        <f t="shared" si="126"/>
+        <f t="shared" si="127"/>
         <v>5884646480.3029652</v>
       </c>
     </row>
@@ -8742,19 +8742,19 @@
         <v>22654230.48</v>
       </c>
       <c r="H181" s="330">
-        <f t="shared" ref="H181:K181" si="127">G181*(1+H190)</f>
+        <f t="shared" ref="H181:K181" si="128">G181*(1+H190)</f>
         <v>22835464.32384</v>
       </c>
       <c r="I181" s="330">
-        <f t="shared" si="127"/>
+        <f t="shared" si="128"/>
         <v>23018148.038430721</v>
       </c>
       <c r="J181" s="330">
-        <f t="shared" si="127"/>
+        <f t="shared" si="128"/>
         <v>23202293.222738165</v>
       </c>
       <c r="K181" s="330">
-        <f t="shared" si="127"/>
+        <f t="shared" si="128"/>
         <v>23387911.568520069</v>
       </c>
     </row>
@@ -8767,31 +8767,31 @@
         <v>1461003005</v>
       </c>
       <c r="E182" s="331">
-        <f t="shared" ref="E182:K182" si="128">SUM(E180:E181)</f>
+        <f t="shared" ref="E182:K182" si="129">SUM(E180:E181)</f>
         <v>2139084215</v>
       </c>
       <c r="F182" s="331">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>2907635027</v>
       </c>
       <c r="G182" s="331">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>3542550152.7199998</v>
       </c>
       <c r="H182" s="331">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>4176312652.5670395</v>
       </c>
       <c r="I182" s="331">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>4799516914.5181103</v>
       </c>
       <c r="J182" s="331">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>5372880911.6799793</v>
       </c>
       <c r="K182" s="331">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>5908034391.8714848</v>
       </c>
     </row>
@@ -8824,19 +8824,19 @@
         <v>-30308823.593999997</v>
       </c>
       <c r="H184" s="330">
-        <f t="shared" ref="H184:K184" si="129">G184*(1+H191)</f>
+        <f t="shared" ref="H184:K184" si="130">G184*(1+H191)</f>
         <v>-30642220.653533995</v>
       </c>
       <c r="I184" s="330">
-        <f t="shared" si="129"/>
+        <f t="shared" si="130"/>
         <v>-30979285.080722865</v>
       </c>
       <c r="J184" s="330">
-        <f t="shared" si="129"/>
+        <f t="shared" si="130"/>
         <v>-31320057.216610812</v>
       </c>
       <c r="K184" s="330">
-        <f t="shared" si="129"/>
+        <f t="shared" si="130"/>
         <v>-31664577.845993526</v>
       </c>
     </row>
@@ -8849,31 +8849,31 @@
         <v>1461003005</v>
       </c>
       <c r="E185" s="331">
-        <f t="shared" ref="E185:K185" si="130">E182+E184</f>
+        <f t="shared" ref="E185:K185" si="131">E182+E184</f>
         <v>2117799758</v>
       </c>
       <c r="F185" s="331">
-        <f t="shared" si="130"/>
+        <f t="shared" si="131"/>
         <v>2877655973</v>
       </c>
       <c r="G185" s="331">
-        <f t="shared" si="130"/>
+        <f t="shared" si="131"/>
         <v>3512241329.1259999</v>
       </c>
       <c r="H185" s="331">
-        <f t="shared" si="130"/>
+        <f t="shared" si="131"/>
         <v>4145670431.9135056</v>
       </c>
       <c r="I185" s="331">
-        <f t="shared" si="130"/>
+        <f t="shared" si="131"/>
         <v>4768537629.4373875</v>
       </c>
       <c r="J185" s="331">
-        <f t="shared" si="130"/>
+        <f t="shared" si="131"/>
         <v>5341560854.4633684</v>
       </c>
       <c r="K185" s="331">
-        <f t="shared" si="130"/>
+        <f t="shared" si="131"/>
         <v>5876369814.0254908</v>
       </c>
     </row>
@@ -8922,7 +8922,7 @@
         <v>0.45209505233016278</v>
       </c>
       <c r="F189" s="1">
-        <f t="shared" ref="F189" si="131">F180/E180-1</f>
+        <f t="shared" ref="F189" si="132">F180/E180-1</f>
         <v>0.35995280373275285</v>
       </c>
       <c r="G189" s="209">
@@ -8976,7 +8976,7 @@
       <c r="D191" s="1"/>
       <c r="E191" s="1"/>
       <c r="F191" s="1">
-        <f t="shared" ref="F191" si="132">F184/E184-1</f>
+        <f t="shared" ref="F191" si="133">F184/E184-1</f>
         <v>0.40849512862836956</v>
       </c>
       <c r="G191" s="209">
@@ -9016,35 +9016,35 @@
         <v>107</v>
       </c>
       <c r="D194" s="48">
-        <f t="shared" ref="D194:K194" si="133">D$13</f>
+        <f t="shared" ref="D194:K194" si="134">D$13</f>
         <v>2023</v>
       </c>
       <c r="E194" s="48">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>2024</v>
       </c>
       <c r="F194" s="48">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>2025</v>
       </c>
       <c r="G194" s="49">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>2026</v>
       </c>
       <c r="H194" s="49">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>2027</v>
       </c>
       <c r="I194" s="49">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>2028</v>
       </c>
       <c r="J194" s="49">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>2029</v>
       </c>
       <c r="K194" s="49">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>2030</v>
       </c>
     </row>
@@ -9053,35 +9053,35 @@
         <v>108</v>
       </c>
       <c r="D195" s="238">
-        <f t="shared" ref="D195:K195" si="134">D$14</f>
+        <f t="shared" ref="D195:K195" si="135">D$14</f>
         <v>45291</v>
       </c>
       <c r="E195" s="224">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>45657</v>
       </c>
       <c r="F195" s="224">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>46022</v>
       </c>
       <c r="G195" s="224">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>46387</v>
       </c>
       <c r="H195" s="224">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>46752</v>
       </c>
       <c r="I195" s="224">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>47118</v>
       </c>
       <c r="J195" s="224">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>47483</v>
       </c>
       <c r="K195" s="224">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>47848</v>
       </c>
     </row>
@@ -9099,15 +9099,15 @@
         <v>321</v>
       </c>
       <c r="D198" s="27">
-        <f>D70</f>
+        <f t="shared" ref="D198:F201" si="136">D70</f>
         <v>138912639</v>
       </c>
       <c r="E198" s="27">
-        <f>E70</f>
+        <f t="shared" si="136"/>
         <v>208473803</v>
       </c>
       <c r="F198" s="27">
-        <f>F70</f>
+        <f t="shared" si="136"/>
         <v>258826409</v>
       </c>
       <c r="G198" s="27">
@@ -9136,15 +9136,15 @@
         <v>341</v>
       </c>
       <c r="D199" s="27">
-        <f>D71</f>
+        <f t="shared" si="136"/>
         <v>16938225</v>
       </c>
       <c r="E199" s="27">
-        <f>E71</f>
+        <f t="shared" si="136"/>
         <v>27584770</v>
       </c>
       <c r="F199" s="27">
-        <f>F71</f>
+        <f t="shared" si="136"/>
         <v>31142087</v>
       </c>
       <c r="G199" s="27">
@@ -9173,15 +9173,15 @@
         <v>342</v>
       </c>
       <c r="D200" s="27">
-        <f>D72</f>
+        <f t="shared" si="136"/>
         <v>39168713</v>
       </c>
       <c r="E200" s="27">
-        <f>E72</f>
+        <f t="shared" si="136"/>
         <v>51382391</v>
       </c>
       <c r="F200" s="27">
-        <f>F72</f>
+        <f t="shared" si="136"/>
         <v>69499941</v>
       </c>
       <c r="G200" s="27">
@@ -9189,19 +9189,19 @@
         <v>84826180.558873415</v>
       </c>
       <c r="H200" s="27">
-        <f t="shared" ref="H200:K201" si="135">$F200/$F$16*H$16</f>
+        <f t="shared" ref="H200:K201" si="137">$F200/$F$16*H$16</f>
         <v>100124494.77171507</v>
       </c>
       <c r="I200" s="27">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>115167722.27524999</v>
       </c>
       <c r="J200" s="27">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>129007139.04521821</v>
       </c>
       <c r="K200" s="27">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>141923620.89175716</v>
       </c>
     </row>
@@ -9210,15 +9210,15 @@
         <v>324</v>
       </c>
       <c r="D201" s="27">
-        <f>D73</f>
+        <f t="shared" si="136"/>
         <v>4251648</v>
       </c>
       <c r="E201" s="27">
-        <f>E73</f>
+        <f t="shared" si="136"/>
         <v>3388601</v>
       </c>
       <c r="F201" s="27">
-        <f>F73</f>
+        <f t="shared" si="136"/>
         <v>0</v>
       </c>
       <c r="G201" s="27">
@@ -9226,19 +9226,19 @@
         <v>0</v>
       </c>
       <c r="H201" s="27">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>0</v>
       </c>
       <c r="I201" s="27">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>0</v>
       </c>
       <c r="J201" s="27">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>0</v>
       </c>
       <c r="K201" s="27">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>0</v>
       </c>
     </row>
@@ -9251,31 +9251,31 @@
         <v>199271225</v>
       </c>
       <c r="E202" s="210">
-        <f t="shared" ref="E202:K202" si="136">SUM(E198:E201)</f>
+        <f t="shared" ref="E202:K202" si="138">SUM(E198:E201)</f>
         <v>290829565</v>
       </c>
       <c r="F202" s="210">
-        <f t="shared" si="136"/>
+        <f t="shared" si="138"/>
         <v>359468437</v>
       </c>
       <c r="G202" s="210">
-        <f t="shared" si="136"/>
+        <f t="shared" si="138"/>
         <v>454664994.11610276</v>
       </c>
       <c r="H202" s="210">
-        <f t="shared" si="136"/>
+        <f t="shared" si="138"/>
         <v>536663357.07128048</v>
       </c>
       <c r="I202" s="210">
-        <f t="shared" si="136"/>
+        <f t="shared" si="138"/>
         <v>617294465.28951347</v>
       </c>
       <c r="J202" s="210">
-        <f t="shared" si="136"/>
+        <f t="shared" si="138"/>
         <v>691473195.28574073</v>
       </c>
       <c r="K202" s="210">
-        <f t="shared" si="136"/>
+        <f t="shared" si="138"/>
         <v>760705030.36384451</v>
       </c>
     </row>
@@ -9359,19 +9359,19 @@
         <v>164181692.73407376</v>
       </c>
       <c r="H206" s="27">
-        <f t="shared" ref="H206:K206" si="137">$F206/$F$16*H$16</f>
+        <f t="shared" ref="H206:K206" si="139">$F206/$F$16*H$16</f>
         <v>193791691.75670853</v>
       </c>
       <c r="I206" s="27">
-        <f t="shared" si="137"/>
+        <f t="shared" si="139"/>
         <v>222907968.58824596</v>
       </c>
       <c r="J206" s="27">
-        <f t="shared" si="137"/>
+        <f t="shared" si="139"/>
         <v>249694260.94251162</v>
       </c>
       <c r="K206" s="27">
-        <f t="shared" si="137"/>
+        <f t="shared" si="139"/>
         <v>274694206.00383461</v>
       </c>
     </row>
@@ -9396,19 +9396,19 @@
         <v>4382238.9367803186</v>
       </c>
       <c r="H207" s="27">
-        <f t="shared" ref="H207:K207" si="138">$F207/$F$16*H$16</f>
+        <f t="shared" ref="H207:K207" si="140">$F207/$F$16*H$16</f>
         <v>5172571.2111903979</v>
       </c>
       <c r="I207" s="27">
-        <f t="shared" si="138"/>
+        <f t="shared" si="140"/>
         <v>5949725.350001134</v>
       </c>
       <c r="J207" s="27">
-        <f t="shared" si="138"/>
+        <f t="shared" si="140"/>
         <v>6664688.9453452965</v>
       </c>
       <c r="K207" s="27">
-        <f t="shared" si="138"/>
+        <f t="shared" si="140"/>
         <v>7331972.4337823819</v>
       </c>
     </row>
@@ -9421,31 +9421,31 @@
         <v>277002298</v>
       </c>
       <c r="E208" s="213">
-        <f t="shared" ref="E208:K208" si="139">SUM(E205:E207)</f>
+        <f t="shared" ref="E208:K208" si="141">SUM(E205:E207)</f>
         <v>321471970</v>
       </c>
       <c r="F208" s="213">
-        <f t="shared" si="139"/>
+        <f t="shared" si="141"/>
         <v>380221750</v>
       </c>
       <c r="G208" s="213">
-        <f t="shared" si="139"/>
+        <f t="shared" si="141"/>
         <v>512580296.81481439</v>
       </c>
       <c r="H208" s="213">
-        <f t="shared" si="139"/>
+        <f t="shared" si="141"/>
         <v>605023624.90433276</v>
       </c>
       <c r="I208" s="213">
-        <f t="shared" si="139"/>
+        <f t="shared" si="141"/>
         <v>695925537.12072682</v>
       </c>
       <c r="J208" s="213">
-        <f t="shared" si="139"/>
+        <f t="shared" si="141"/>
         <v>779553166.10221541</v>
       </c>
       <c r="K208" s="213">
-        <f t="shared" si="139"/>
+        <f t="shared" si="141"/>
         <v>857603763.86674631</v>
       </c>
     </row>
@@ -9463,35 +9463,35 @@
         <v>163</v>
       </c>
       <c r="D210" s="19">
-        <f t="shared" ref="D210:K210" si="140">D202-D208</f>
+        <f t="shared" ref="D210:K210" si="142">D202-D208</f>
         <v>-77731073</v>
       </c>
       <c r="E210" s="19">
-        <f t="shared" si="140"/>
+        <f t="shared" si="142"/>
         <v>-30642405</v>
       </c>
       <c r="F210" s="19">
-        <f t="shared" si="140"/>
+        <f t="shared" si="142"/>
         <v>-20753313</v>
       </c>
       <c r="G210" s="19">
-        <f t="shared" si="140"/>
+        <f t="shared" si="142"/>
         <v>-57915302.698711634</v>
       </c>
       <c r="H210" s="19">
-        <f t="shared" si="140"/>
+        <f t="shared" si="142"/>
         <v>-68360267.833052278</v>
       </c>
       <c r="I210" s="19">
-        <f t="shared" si="140"/>
+        <f t="shared" si="142"/>
         <v>-78631071.831213355</v>
       </c>
       <c r="J210" s="19">
-        <f t="shared" si="140"/>
+        <f t="shared" si="142"/>
         <v>-88079970.816474676</v>
       </c>
       <c r="K210" s="19">
-        <f t="shared" si="140"/>
+        <f t="shared" si="142"/>
         <v>-96898733.502901793</v>
       </c>
     </row>
@@ -9500,35 +9500,35 @@
         <v>164</v>
       </c>
       <c r="D211" s="22">
-        <f>D210/D16</f>
+        <f t="shared" ref="D211:K211" si="143">D210/D16</f>
         <v>-5.320391041906173E-2</v>
       </c>
       <c r="E211" s="22">
-        <f>E210/E16</f>
+        <f t="shared" si="143"/>
         <v>-1.4468981254836841E-2</v>
       </c>
       <c r="F211" s="22">
-        <f>F210/F16</f>
+        <f t="shared" si="143"/>
         <v>-7.2118811959180637E-3</v>
       </c>
       <c r="G211" s="22">
-        <f>G210/G16</f>
+        <f t="shared" si="143"/>
         <v>-1.648955674498697E-2</v>
       </c>
       <c r="H211" s="22">
-        <f>H210/H16</f>
+        <f t="shared" si="143"/>
         <v>-1.6489556744986943E-2</v>
       </c>
       <c r="I211" s="22">
-        <f>I210/I16</f>
+        <f t="shared" si="143"/>
         <v>-1.648955674498695E-2</v>
       </c>
       <c r="J211" s="22">
-        <f>J210/J16</f>
+        <f t="shared" si="143"/>
         <v>-1.6489556744986946E-2</v>
       </c>
       <c r="K211" s="22">
-        <f>K210/K16</f>
+        <f t="shared" si="143"/>
         <v>-1.648955674498696E-2</v>
       </c>
     </row>
@@ -9542,27 +9542,27 @@
         <v>-47088668</v>
       </c>
       <c r="F212" s="183">
-        <f t="shared" ref="F212:K212" si="141">E210-F210</f>
+        <f t="shared" ref="F212:K212" si="144">E210-F210</f>
         <v>-9889092</v>
       </c>
       <c r="G212" s="183">
-        <f t="shared" si="141"/>
+        <f t="shared" si="144"/>
         <v>37161989.698711634</v>
       </c>
       <c r="H212" s="183">
-        <f t="shared" si="141"/>
+        <f t="shared" si="144"/>
         <v>10444965.134340644</v>
       </c>
       <c r="I212" s="183">
-        <f t="shared" si="141"/>
+        <f t="shared" si="144"/>
         <v>10270803.998161077</v>
       </c>
       <c r="J212" s="183">
-        <f t="shared" si="141"/>
+        <f t="shared" si="144"/>
         <v>9448898.9852613211</v>
       </c>
       <c r="K212" s="183">
-        <f t="shared" si="141"/>
+        <f t="shared" si="144"/>
         <v>8818762.6864271164</v>
       </c>
     </row>
@@ -9591,35 +9591,35 @@
         <v>321</v>
       </c>
       <c r="D215" s="333">
-        <f>-D17/AVERAGE(D198:E198)</f>
+        <f t="shared" ref="D215:K215" si="145">-D17/AVERAGE(D198:E198)</f>
         <v>5.6929976674219196</v>
       </c>
       <c r="E215" s="333">
-        <f>-E17/AVERAGE(E198:F198)</f>
+        <f t="shared" si="145"/>
         <v>6.1031672975145153</v>
       </c>
       <c r="F215" s="333">
-        <f>-F17/AVERAGE(F198:G198)</f>
+        <f t="shared" si="145"/>
         <v>6.5132434382810862</v>
       </c>
       <c r="G215" s="333">
-        <f>-G17/AVERAGE(G198:H198)</f>
+        <f t="shared" si="145"/>
         <v>6.5328599686121569</v>
       </c>
       <c r="H215" s="333">
-        <f>-H17/AVERAGE(H198:I198)</f>
+        <f t="shared" si="145"/>
         <v>6.6243209448131717</v>
       </c>
       <c r="I215" s="333">
-        <f>-I17/AVERAGE(I198:J198)</f>
+        <f t="shared" si="145"/>
         <v>6.7182967980235011</v>
       </c>
       <c r="J215" s="333">
-        <f>-J17/AVERAGE(J198:K198)</f>
+        <f t="shared" si="145"/>
         <v>6.7824216732056826</v>
       </c>
       <c r="K215" s="333">
-        <f>-K17/AVERAGE(K198:L198)</f>
+        <f t="shared" si="145"/>
         <v>7.1219572487788581</v>
       </c>
     </row>
@@ -9628,35 +9628,35 @@
         <v>341</v>
       </c>
       <c r="D216" s="333">
-        <f>D16/AVERAGE(D199:E199)</f>
+        <f t="shared" ref="D216:K216" si="146">D16/AVERAGE(D199:E199)</f>
         <v>65.629143097853145</v>
       </c>
       <c r="E216" s="333">
-        <f>E16/AVERAGE(E199:F199)</f>
+        <f t="shared" si="146"/>
         <v>72.123722132788416</v>
       </c>
       <c r="F216" s="333">
-        <f>F16/AVERAGE(F199:G199)</f>
+        <f t="shared" si="146"/>
         <v>83.227365652909924</v>
       </c>
       <c r="G216" s="333">
-        <f>G16/AVERAGE(G199:H199)</f>
+        <f t="shared" si="146"/>
         <v>84.7608192111948</v>
       </c>
       <c r="H216" s="333">
-        <f>H16/AVERAGE(H199:I199)</f>
+        <f t="shared" si="146"/>
         <v>85.947482832625596</v>
       </c>
       <c r="I216" s="333">
-        <f>I16/AVERAGE(I199:J199)</f>
+        <f t="shared" si="146"/>
         <v>87.166775813410354</v>
       </c>
       <c r="J216" s="333">
-        <f>J16/AVERAGE(J199:K199)</f>
+        <f t="shared" si="146"/>
         <v>87.998766240018568</v>
       </c>
       <c r="K216" s="333">
-        <f>K16/AVERAGE(K199:L199)</f>
+        <f t="shared" si="146"/>
         <v>92.404082391780619</v>
       </c>
     </row>
@@ -9665,35 +9665,35 @@
         <v>343</v>
       </c>
       <c r="D217" s="333">
-        <f>-D19/AVERAGE(D205:E205)</f>
+        <f t="shared" ref="D217:K217" si="147">-D19/AVERAGE(D205:E205)</f>
         <v>1.6751979580136303</v>
       </c>
       <c r="E217" s="333">
-        <f>-E19/AVERAGE(E205:F205)</f>
+        <f t="shared" si="147"/>
         <v>1.7726495940560534</v>
       </c>
       <c r="F217" s="333">
-        <f>-F19/AVERAGE(F205:G205)</f>
+        <f t="shared" si="147"/>
         <v>2.0212408468434235</v>
       </c>
       <c r="G217" s="333">
-        <f>-G19/AVERAGE(G205:H205)</f>
+        <f t="shared" si="147"/>
         <v>1.8440505418520825</v>
       </c>
       <c r="H217" s="333">
-        <f>-H19/AVERAGE(H205:I205)</f>
+        <f t="shared" si="147"/>
         <v>1.8681572367269839</v>
       </c>
       <c r="I217" s="333">
-        <f>-I19/AVERAGE(I205:J205)</f>
+        <f t="shared" si="147"/>
         <v>1.8934035640607243</v>
       </c>
       <c r="J217" s="333">
-        <f>-J19/AVERAGE(J205:K205)</f>
+        <f t="shared" si="147"/>
         <v>1.9105701991976041</v>
       </c>
       <c r="K217" s="333">
-        <f>-K19/AVERAGE(K205:L205)</f>
+        <f t="shared" si="147"/>
         <v>2.0054953125801691</v>
       </c>
     </row>
@@ -9743,15 +9743,15 @@
         <v>51.24995661306216</v>
       </c>
       <c r="I220" s="249">
-        <f t="shared" ref="I220:K220" si="142">H220</f>
+        <f t="shared" ref="I220:K220" si="148">H220</f>
         <v>51.24995661306216</v>
       </c>
       <c r="J220" s="249">
-        <f t="shared" si="142"/>
+        <f t="shared" si="148"/>
         <v>51.24995661306216</v>
       </c>
       <c r="K220" s="249">
-        <f t="shared" si="142"/>
+        <f t="shared" si="148"/>
         <v>51.24995661306216</v>
       </c>
     </row>
@@ -9780,15 +9780,15 @@
         <v>3.950041930533438</v>
       </c>
       <c r="I221" s="249">
-        <f t="shared" ref="I221:K221" si="143">H221</f>
+        <f t="shared" ref="I221:K221" si="149">H221</f>
         <v>3.950041930533438</v>
       </c>
       <c r="J221" s="249">
-        <f t="shared" si="143"/>
+        <f t="shared" si="149"/>
         <v>3.950041930533438</v>
       </c>
       <c r="K221" s="249">
-        <f t="shared" si="143"/>
+        <f t="shared" si="149"/>
         <v>3.950041930533438</v>
       </c>
     </row>
@@ -9817,15 +9817,15 @@
         <v>53.132221519200364</v>
       </c>
       <c r="I222" s="249">
-        <f t="shared" ref="I222:K222" si="144">H222</f>
+        <f t="shared" ref="I222:K222" si="150">H222</f>
         <v>53.132221519200364</v>
       </c>
       <c r="J222" s="249">
-        <f t="shared" si="144"/>
+        <f t="shared" si="150"/>
         <v>53.132221519200364</v>
       </c>
       <c r="K222" s="249">
-        <f t="shared" si="144"/>
+        <f t="shared" si="150"/>
         <v>53.132221519200364</v>
       </c>
     </row>
@@ -9850,35 +9850,35 @@
         <v>107</v>
       </c>
       <c r="D225" s="48">
-        <f t="shared" ref="D225:K225" si="145">D$13</f>
+        <f t="shared" ref="D225:K225" si="151">D$13</f>
         <v>2023</v>
       </c>
       <c r="E225" s="48">
-        <f t="shared" si="145"/>
+        <f t="shared" si="151"/>
         <v>2024</v>
       </c>
       <c r="F225" s="48">
-        <f t="shared" si="145"/>
+        <f t="shared" si="151"/>
         <v>2025</v>
       </c>
       <c r="G225" s="49">
-        <f t="shared" si="145"/>
+        <f t="shared" si="151"/>
         <v>2026</v>
       </c>
       <c r="H225" s="49">
-        <f t="shared" si="145"/>
+        <f t="shared" si="151"/>
         <v>2027</v>
       </c>
       <c r="I225" s="49">
-        <f t="shared" si="145"/>
+        <f t="shared" si="151"/>
         <v>2028</v>
       </c>
       <c r="J225" s="49">
-        <f t="shared" si="145"/>
+        <f t="shared" si="151"/>
         <v>2029</v>
       </c>
       <c r="K225" s="49">
-        <f t="shared" si="145"/>
+        <f t="shared" si="151"/>
         <v>2030</v>
       </c>
     </row>
@@ -9887,35 +9887,35 @@
         <v>108</v>
       </c>
       <c r="D226" s="238">
-        <f t="shared" ref="D226:K226" si="146">D$14</f>
+        <f t="shared" ref="D226:K226" si="152">D$14</f>
         <v>45291</v>
       </c>
       <c r="E226" s="224">
-        <f t="shared" si="146"/>
+        <f t="shared" si="152"/>
         <v>45657</v>
       </c>
       <c r="F226" s="224">
-        <f t="shared" si="146"/>
+        <f t="shared" si="152"/>
         <v>46022</v>
       </c>
       <c r="G226" s="224">
-        <f t="shared" si="146"/>
+        <f t="shared" si="152"/>
         <v>46387</v>
       </c>
       <c r="H226" s="224">
-        <f t="shared" si="146"/>
+        <f t="shared" si="152"/>
         <v>46752</v>
       </c>
       <c r="I226" s="224">
-        <f t="shared" si="146"/>
+        <f t="shared" si="152"/>
         <v>47118</v>
       </c>
       <c r="J226" s="224">
-        <f t="shared" si="146"/>
+        <f t="shared" si="152"/>
         <v>47483</v>
       </c>
       <c r="K226" s="224">
-        <f t="shared" si="146"/>
+        <f t="shared" si="152"/>
         <v>47848</v>
       </c>
     </row>
@@ -9942,27 +9942,27 @@
         <v>127986330</v>
       </c>
       <c r="F229" s="183">
-        <f t="shared" ref="F229:K229" si="147">E232</f>
+        <f t="shared" ref="F229:K229" si="153">E232</f>
         <v>50000047</v>
       </c>
       <c r="G229" s="183">
-        <f t="shared" si="147"/>
+        <f t="shared" si="153"/>
         <v>22377172</v>
       </c>
       <c r="H229" s="183">
-        <f t="shared" si="147"/>
+        <f t="shared" si="153"/>
         <v>6441727</v>
       </c>
       <c r="I229" s="183">
-        <f t="shared" si="147"/>
+        <f t="shared" si="153"/>
         <v>0</v>
       </c>
       <c r="J229" s="183">
-        <f t="shared" si="147"/>
+        <f t="shared" si="153"/>
         <v>0</v>
       </c>
       <c r="K229" s="183">
-        <f t="shared" si="147"/>
+        <f t="shared" si="153"/>
         <v>0</v>
       </c>
     </row>
@@ -9979,23 +9979,23 @@
         <v>0</v>
       </c>
       <c r="G230" s="183">
-        <f t="shared" ref="G230:K230" si="148">F230</f>
+        <f t="shared" ref="G230:K230" si="154">F230</f>
         <v>0</v>
       </c>
       <c r="H230" s="183">
-        <f t="shared" si="148"/>
+        <f t="shared" si="154"/>
         <v>0</v>
       </c>
       <c r="I230" s="183">
-        <f t="shared" si="148"/>
+        <f t="shared" si="154"/>
         <v>0</v>
       </c>
       <c r="J230" s="183">
-        <f t="shared" si="148"/>
+        <f t="shared" si="154"/>
         <v>0</v>
       </c>
       <c r="K230" s="183">
-        <f t="shared" si="148"/>
+        <f t="shared" si="154"/>
         <v>0</v>
       </c>
     </row>
@@ -10043,19 +10043,19 @@
         <v>6441727</v>
       </c>
       <c r="H232" s="19">
-        <f t="shared" ref="H232:K232" si="149">H229+H230-H231</f>
+        <f t="shared" ref="H232:K232" si="155">H229+H230-H231</f>
         <v>0</v>
       </c>
       <c r="I232" s="19">
-        <f t="shared" si="149"/>
+        <f t="shared" si="155"/>
         <v>0</v>
       </c>
       <c r="J232" s="19">
-        <f t="shared" si="149"/>
+        <f t="shared" si="155"/>
         <v>0</v>
       </c>
       <c r="K232" s="19">
-        <f t="shared" si="149"/>
+        <f t="shared" si="155"/>
         <v>0</v>
       </c>
     </row>
@@ -10069,27 +10069,27 @@
         <v>88993188.5</v>
       </c>
       <c r="F233" s="183">
-        <f t="shared" ref="F233:K233" si="150">AVERAGE(F229,F232)</f>
+        <f t="shared" ref="F233:K233" si="156">AVERAGE(F229,F232)</f>
         <v>36188609.5</v>
       </c>
       <c r="G233" s="183">
-        <f t="shared" si="150"/>
+        <f t="shared" si="156"/>
         <v>14409449.5</v>
       </c>
       <c r="H233" s="183">
-        <f t="shared" si="150"/>
+        <f t="shared" si="156"/>
         <v>3220863.5</v>
       </c>
       <c r="I233" s="183">
-        <f t="shared" si="150"/>
+        <f t="shared" si="156"/>
         <v>0</v>
       </c>
       <c r="J233" s="183">
-        <f t="shared" si="150"/>
+        <f t="shared" si="156"/>
         <v>0</v>
       </c>
       <c r="K233" s="183">
-        <f t="shared" si="150"/>
+        <f t="shared" si="156"/>
         <v>0</v>
       </c>
     </row>
@@ -10103,7 +10103,7 @@
         <v>0.62500199102316689</v>
       </c>
       <c r="F234" s="1">
-        <f t="shared" ref="F234" si="151">-F241/F233</f>
+        <f t="shared" ref="F234" si="157">-F241/F233</f>
         <v>1.0439991345895729</v>
       </c>
       <c r="G234" s="209">
@@ -10114,15 +10114,15 @@
         <v>0.2</v>
       </c>
       <c r="I234" s="209">
-        <f t="shared" ref="I234:K234" si="152">H234</f>
+        <f t="shared" ref="I234:K234" si="158">H234</f>
         <v>0.2</v>
       </c>
       <c r="J234" s="209">
-        <f t="shared" si="152"/>
+        <f t="shared" si="158"/>
         <v>0.2</v>
       </c>
       <c r="K234" s="209">
-        <f t="shared" si="152"/>
+        <f t="shared" si="158"/>
         <v>0.2</v>
       </c>
     </row>
@@ -10148,35 +10148,35 @@
         <v>174</v>
       </c>
       <c r="D237" s="183">
-        <f>D69+D74</f>
+        <f t="shared" ref="D237:K237" si="159">D69+D74</f>
         <v>71703738</v>
       </c>
       <c r="E237" s="183">
-        <f>E69+E74</f>
+        <f t="shared" si="159"/>
         <v>93205257</v>
       </c>
       <c r="F237" s="183">
-        <f>F69+F74</f>
+        <f t="shared" si="159"/>
         <v>306003759</v>
       </c>
       <c r="G237" s="183">
-        <f>G69+G74</f>
+        <f t="shared" si="159"/>
         <v>364339486.62656695</v>
       </c>
       <c r="H237" s="183">
-        <f>H69+H74</f>
+        <f t="shared" si="159"/>
         <v>498607483.70045131</v>
       </c>
       <c r="I237" s="183">
-        <f>I69+I74</f>
+        <f t="shared" si="159"/>
         <v>650795449.00696623</v>
       </c>
       <c r="J237" s="183">
-        <f>J69+J74</f>
+        <f t="shared" si="159"/>
         <v>813582368.17115283</v>
       </c>
       <c r="K237" s="183">
-        <f>K69+K74</f>
+        <f t="shared" si="159"/>
         <v>996491174.74343967</v>
       </c>
     </row>
@@ -10190,27 +10190,27 @@
         <v>82454497.5</v>
       </c>
       <c r="F238" s="183">
-        <f t="shared" ref="F238" si="153">AVERAGE(E237,F237)</f>
+        <f t="shared" ref="F238" si="160">AVERAGE(E237,F237)</f>
         <v>199604508</v>
       </c>
       <c r="G238" s="183">
-        <f t="shared" ref="G238" si="154">AVERAGE(F237,G237)</f>
+        <f t="shared" ref="G238" si="161">AVERAGE(F237,G237)</f>
         <v>335171622.81328344</v>
       </c>
       <c r="H238" s="183">
-        <f t="shared" ref="H238" si="155">AVERAGE(G237,H237)</f>
+        <f t="shared" ref="H238" si="162">AVERAGE(G237,H237)</f>
         <v>431473485.16350913</v>
       </c>
       <c r="I238" s="183">
-        <f t="shared" ref="I238" si="156">AVERAGE(H237,I237)</f>
+        <f t="shared" ref="I238" si="163">AVERAGE(H237,I237)</f>
         <v>574701466.35370874</v>
       </c>
       <c r="J238" s="183">
-        <f t="shared" ref="J238" si="157">AVERAGE(I237,J237)</f>
+        <f t="shared" ref="J238" si="164">AVERAGE(I237,J237)</f>
         <v>732188908.58905959</v>
       </c>
       <c r="K238" s="183">
-        <f t="shared" ref="K238" si="158">AVERAGE(J237,K237)</f>
+        <f t="shared" ref="K238" si="165">AVERAGE(J237,K237)</f>
         <v>905036771.45729625</v>
       </c>
     </row>
@@ -10224,7 +10224,7 @@
         <v>0.10288512157872286</v>
       </c>
       <c r="F239" s="1">
-        <f t="shared" ref="F239" si="159">F242/F238</f>
+        <f t="shared" ref="F239" si="166">F242/F238</f>
         <v>0.180557525283948</v>
       </c>
       <c r="G239" s="209">
@@ -10240,7 +10240,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="K239" s="209">
-        <f t="shared" ref="K239" si="160">J239</f>
+        <f t="shared" ref="K239" si="167">J239</f>
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
@@ -10260,15 +10260,15 @@
         <v>223</v>
       </c>
       <c r="D241" s="231">
-        <f>D26</f>
+        <f t="shared" ref="D241:F242" si="168">D26</f>
         <v>-47950964</v>
       </c>
       <c r="E241" s="231">
-        <f>E26</f>
+        <f t="shared" si="168"/>
         <v>-55620920</v>
       </c>
       <c r="F241" s="231">
-        <f>F26</f>
+        <f t="shared" si="168"/>
         <v>-37780877</v>
       </c>
       <c r="G241" s="19">
@@ -10276,19 +10276,19 @@
         <v>-40228350.490431122</v>
       </c>
       <c r="H241" s="19">
-        <f t="shared" ref="H241:I241" si="161">-(H234*G233)-H270</f>
+        <f t="shared" ref="H241:I241" si="169">-(H234*G233)-H270</f>
         <v>-41822344.345260054</v>
       </c>
       <c r="I241" s="19">
-        <f t="shared" si="161"/>
+        <f t="shared" si="169"/>
         <v>-45435244.585544705</v>
       </c>
       <c r="J241" s="19">
-        <f t="shared" ref="J241" si="162">-(J234*I233)-J270</f>
+        <f t="shared" ref="J241" si="170">-(J234*I233)-J270</f>
         <v>-50173502.823235251</v>
       </c>
       <c r="K241" s="19">
-        <f t="shared" ref="K241" si="163">-(K234*J233)-K270</f>
+        <f t="shared" ref="K241" si="171">-(K234*J233)-K270</f>
         <v>-55196985.57922782</v>
       </c>
     </row>
@@ -10297,15 +10297,15 @@
         <v>109</v>
       </c>
       <c r="D242" s="231">
-        <f>D27</f>
+        <f t="shared" si="168"/>
         <v>-435610</v>
       </c>
       <c r="E242" s="231">
-        <f>E27</f>
+        <f t="shared" si="168"/>
         <v>8483341</v>
       </c>
       <c r="F242" s="231">
-        <f>F27</f>
+        <f t="shared" si="168"/>
         <v>36040096</v>
       </c>
       <c r="G242" s="183">
@@ -10313,19 +10313,19 @@
         <v>42840526.260000005</v>
       </c>
       <c r="H242" s="183">
-        <f t="shared" ref="H242:K242" si="164">H239*G237</f>
+        <f t="shared" ref="H242:K242" si="172">H239*G237</f>
         <v>43720738.395188034</v>
       </c>
       <c r="I242" s="183">
-        <f t="shared" si="164"/>
+        <f t="shared" si="172"/>
         <v>49860748.370045133</v>
       </c>
       <c r="J242" s="183">
-        <f t="shared" si="164"/>
+        <f t="shared" si="172"/>
         <v>55317613.165592134</v>
       </c>
       <c r="K242" s="183">
-        <f t="shared" si="164"/>
+        <f t="shared" si="172"/>
         <v>69154501.29454799</v>
       </c>
     </row>
@@ -10338,31 +10338,31 @@
         <v>-48386574</v>
       </c>
       <c r="E243" s="183">
-        <f t="shared" ref="E243:F243" si="165">SUM(E241:E242)</f>
+        <f t="shared" ref="E243:F243" si="173">SUM(E241:E242)</f>
         <v>-47137579</v>
       </c>
       <c r="F243" s="183">
-        <f t="shared" si="165"/>
+        <f t="shared" si="173"/>
         <v>-1740781</v>
       </c>
       <c r="G243" s="183">
-        <f t="shared" ref="G243" si="166">SUM(G241:G242)</f>
+        <f t="shared" ref="G243" si="174">SUM(G241:G242)</f>
         <v>2612175.7695688829</v>
       </c>
       <c r="H243" s="183">
-        <f t="shared" ref="H243" si="167">SUM(H241:H242)</f>
+        <f t="shared" ref="H243" si="175">SUM(H241:H242)</f>
         <v>1898394.0499279797</v>
       </c>
       <c r="I243" s="183">
-        <f t="shared" ref="I243" si="168">SUM(I241:I242)</f>
+        <f t="shared" ref="I243" si="176">SUM(I241:I242)</f>
         <v>4425503.7845004275</v>
       </c>
       <c r="J243" s="183">
-        <f t="shared" ref="J243" si="169">SUM(J241:J242)</f>
+        <f t="shared" ref="J243" si="177">SUM(J241:J242)</f>
         <v>5144110.342356883</v>
       </c>
       <c r="K243" s="183">
-        <f t="shared" ref="K243" si="170">SUM(K241:K242)</f>
+        <f t="shared" ref="K243" si="178">SUM(K241:K242)</f>
         <v>13957515.71532017</v>
       </c>
     </row>
@@ -10376,35 +10376,35 @@
         <v>107</v>
       </c>
       <c r="D246" s="48">
-        <f t="shared" ref="D246:K246" si="171">D$13</f>
+        <f t="shared" ref="D246:K246" si="179">D$13</f>
         <v>2023</v>
       </c>
       <c r="E246" s="48">
-        <f t="shared" si="171"/>
+        <f t="shared" si="179"/>
         <v>2024</v>
       </c>
       <c r="F246" s="48">
-        <f t="shared" si="171"/>
+        <f t="shared" si="179"/>
         <v>2025</v>
       </c>
       <c r="G246" s="49">
-        <f t="shared" si="171"/>
+        <f t="shared" si="179"/>
         <v>2026</v>
       </c>
       <c r="H246" s="49">
-        <f t="shared" si="171"/>
+        <f t="shared" si="179"/>
         <v>2027</v>
       </c>
       <c r="I246" s="49">
-        <f t="shared" si="171"/>
+        <f t="shared" si="179"/>
         <v>2028</v>
       </c>
       <c r="J246" s="49">
-        <f t="shared" si="171"/>
+        <f t="shared" si="179"/>
         <v>2029</v>
       </c>
       <c r="K246" s="49">
-        <f t="shared" si="171"/>
+        <f t="shared" si="179"/>
         <v>2030</v>
       </c>
     </row>
@@ -10413,35 +10413,35 @@
         <v>108</v>
       </c>
       <c r="D247" s="238">
-        <f t="shared" ref="D247:K247" si="172">D$14</f>
+        <f t="shared" ref="D247:K247" si="180">D$14</f>
         <v>45291</v>
       </c>
       <c r="E247" s="224">
-        <f t="shared" si="172"/>
+        <f t="shared" si="180"/>
         <v>45657</v>
       </c>
       <c r="F247" s="224">
-        <f t="shared" si="172"/>
+        <f t="shared" si="180"/>
         <v>46022</v>
       </c>
       <c r="G247" s="224">
-        <f t="shared" si="172"/>
+        <f t="shared" si="180"/>
         <v>46387</v>
       </c>
       <c r="H247" s="224">
-        <f t="shared" si="172"/>
+        <f t="shared" si="180"/>
         <v>46752</v>
       </c>
       <c r="I247" s="224">
-        <f t="shared" si="172"/>
+        <f t="shared" si="180"/>
         <v>47118</v>
       </c>
       <c r="J247" s="224">
-        <f t="shared" si="172"/>
+        <f t="shared" si="180"/>
         <v>47483</v>
       </c>
       <c r="K247" s="224">
-        <f t="shared" si="172"/>
+        <f t="shared" si="180"/>
         <v>47848</v>
       </c>
     </row>
@@ -10460,27 +10460,27 @@
         <v>-83822569</v>
       </c>
       <c r="F250" s="183">
-        <f t="shared" ref="F250:K250" si="173">E253</f>
+        <f t="shared" ref="F250:K250" si="181">E253</f>
         <v>-53757977</v>
       </c>
       <c r="G250" s="183">
-        <f t="shared" si="173"/>
+        <f t="shared" si="181"/>
         <v>151119171</v>
       </c>
       <c r="H250" s="183">
-        <f t="shared" si="173"/>
+        <f t="shared" si="181"/>
         <v>303078648.68594241</v>
       </c>
       <c r="I250" s="183">
-        <f t="shared" si="173"/>
+        <f t="shared" si="181"/>
         <v>463664114.48953038</v>
       </c>
       <c r="J250" s="183">
-        <f t="shared" si="173"/>
+        <f t="shared" si="181"/>
         <v>637737493.03175485</v>
       </c>
       <c r="K250" s="183">
-        <f t="shared" si="173"/>
+        <f t="shared" si="181"/>
         <v>823685600.51448762</v>
       </c>
     </row>
@@ -10489,35 +10489,35 @@
         <v>226</v>
       </c>
       <c r="D251" s="255">
-        <f>D32</f>
+        <f t="shared" ref="D251:K251" si="182">D32</f>
         <v>31745161</v>
       </c>
       <c r="E251" s="255">
-        <f>E32</f>
+        <f t="shared" si="182"/>
         <v>135031718</v>
       </c>
       <c r="F251" s="255">
-        <f>F32</f>
+        <f t="shared" si="182"/>
         <v>211202869</v>
       </c>
       <c r="G251" s="255">
-        <f>G32</f>
+        <f t="shared" si="182"/>
         <v>289241342.53594244</v>
       </c>
       <c r="H251" s="255">
-        <f>H32</f>
+        <f t="shared" si="182"/>
         <v>348592338.45195049</v>
       </c>
       <c r="I251" s="255">
-        <f>I32</f>
+        <f t="shared" si="182"/>
         <v>400658398.53599232</v>
       </c>
       <c r="J251" s="255">
-        <f>J32</f>
+        <f t="shared" si="182"/>
         <v>446376066.53112787</v>
       </c>
       <c r="K251" s="255">
-        <f>K32</f>
+        <f t="shared" si="182"/>
         <v>494736104.12427253</v>
       </c>
     </row>
@@ -10539,19 +10539,19 @@
         <v>137281864.84999999</v>
       </c>
       <c r="H252" s="183">
-        <f t="shared" ref="H252:K252" si="174">H261*G251</f>
+        <f t="shared" ref="H252:K252" si="183">H261*G251</f>
         <v>188006872.64836258</v>
       </c>
       <c r="I252" s="183">
-        <f t="shared" si="174"/>
+        <f t="shared" si="183"/>
         <v>226585019.99376783</v>
       </c>
       <c r="J252" s="183">
-        <f t="shared" si="174"/>
+        <f t="shared" si="183"/>
         <v>260427959.04839501</v>
       </c>
       <c r="K252" s="183">
-        <f t="shared" si="174"/>
+        <f t="shared" si="183"/>
         <v>290144443.24523312</v>
       </c>
     </row>
@@ -10576,19 +10576,19 @@
         <v>303078648.68594241</v>
       </c>
       <c r="H253" s="19">
-        <f t="shared" ref="H253:K253" si="175">H250+H251-H252</f>
+        <f t="shared" ref="H253:K253" si="184">H250+H251-H252</f>
         <v>463664114.48953038</v>
       </c>
       <c r="I253" s="19">
-        <f t="shared" si="175"/>
+        <f t="shared" si="184"/>
         <v>637737493.03175485</v>
       </c>
       <c r="J253" s="19">
-        <f t="shared" si="175"/>
+        <f t="shared" si="184"/>
         <v>823685600.51448762</v>
       </c>
       <c r="K253" s="19">
-        <f t="shared" si="175"/>
+        <f t="shared" si="184"/>
         <v>1028277261.393527</v>
       </c>
     </row>
@@ -10626,27 +10626,27 @@
         <v>-436852</v>
       </c>
       <c r="F256" s="183">
-        <f t="shared" ref="F256:K256" si="176">E259</f>
+        <f t="shared" ref="F256:K256" si="185">E259</f>
         <v>-426786</v>
       </c>
       <c r="G256" s="183">
-        <f t="shared" si="176"/>
+        <f t="shared" si="185"/>
         <v>-417023</v>
       </c>
       <c r="H256" s="183">
-        <f t="shared" si="176"/>
+        <f t="shared" si="185"/>
         <v>-403652.61710440397</v>
       </c>
       <c r="I256" s="183">
-        <f t="shared" si="176"/>
+        <f t="shared" si="185"/>
         <v>-387538.69300659071</v>
       </c>
       <c r="J256" s="183">
-        <f t="shared" si="176"/>
+        <f t="shared" si="185"/>
         <v>-369017.97894892847</v>
       </c>
       <c r="K256" s="183">
-        <f t="shared" si="176"/>
+        <f t="shared" si="185"/>
         <v>-348383.93378572853</v>
       </c>
     </row>
@@ -10727,19 +10727,19 @@
         <v>-403652.61710440397</v>
       </c>
       <c r="H259" s="183">
-        <f t="shared" ref="H259:K259" si="177">H256+H257-H258</f>
+        <f t="shared" ref="H259:K259" si="186">H256+H257-H258</f>
         <v>-387538.69300659071</v>
       </c>
       <c r="I259" s="183">
-        <f t="shared" si="177"/>
+        <f t="shared" si="186"/>
         <v>-369017.97894892847</v>
       </c>
       <c r="J259" s="183">
-        <f t="shared" si="177"/>
+        <f t="shared" si="186"/>
         <v>-348383.93378572853</v>
       </c>
       <c r="K259" s="183">
-        <f t="shared" si="177"/>
+        <f t="shared" si="186"/>
         <v>-325514.41213843843</v>
       </c>
     </row>
@@ -10771,15 +10771,15 @@
         <v>0.65</v>
       </c>
       <c r="I261" s="209">
-        <f t="shared" ref="I261:K261" si="178">H261</f>
+        <f t="shared" ref="I261:K261" si="187">H261</f>
         <v>0.65</v>
       </c>
       <c r="J261" s="209">
-        <f t="shared" si="178"/>
+        <f t="shared" si="187"/>
         <v>0.65</v>
       </c>
       <c r="K261" s="209">
-        <f t="shared" si="178"/>
+        <f t="shared" si="187"/>
         <v>0.65</v>
       </c>
     </row>
@@ -10808,15 +10808,15 @@
         <v>4.6223561098372186E-5</v>
       </c>
       <c r="I262" s="209">
-        <f t="shared" ref="I262:K262" si="179">H262</f>
+        <f t="shared" ref="I262:K262" si="188">H262</f>
         <v>4.6223561098372186E-5</v>
       </c>
       <c r="J262" s="209">
-        <f t="shared" si="179"/>
+        <f t="shared" si="188"/>
         <v>4.6223561098372186E-5</v>
       </c>
       <c r="K262" s="209">
-        <f t="shared" si="179"/>
+        <f t="shared" si="188"/>
         <v>4.6223561098372186E-5</v>
       </c>
     </row>
@@ -10840,35 +10840,35 @@
         <v>107</v>
       </c>
       <c r="D265" s="48">
-        <f t="shared" ref="D265:K265" si="180">D$13</f>
+        <f t="shared" ref="D265:K265" si="189">D$13</f>
         <v>2023</v>
       </c>
       <c r="E265" s="48">
-        <f t="shared" si="180"/>
+        <f t="shared" si="189"/>
         <v>2024</v>
       </c>
       <c r="F265" s="48">
-        <f t="shared" si="180"/>
+        <f t="shared" si="189"/>
         <v>2025</v>
       </c>
       <c r="G265" s="49">
-        <f t="shared" si="180"/>
+        <f t="shared" si="189"/>
         <v>2026</v>
       </c>
       <c r="H265" s="49">
-        <f t="shared" si="180"/>
+        <f t="shared" si="189"/>
         <v>2027</v>
       </c>
       <c r="I265" s="49">
-        <f t="shared" si="180"/>
+        <f t="shared" si="189"/>
         <v>2028</v>
       </c>
       <c r="J265" s="49">
-        <f t="shared" si="180"/>
+        <f t="shared" si="189"/>
         <v>2029</v>
       </c>
       <c r="K265" s="49">
-        <f t="shared" si="180"/>
+        <f t="shared" si="189"/>
         <v>2030</v>
       </c>
     </row>
@@ -10877,35 +10877,35 @@
         <v>108</v>
       </c>
       <c r="D266" s="238">
-        <f t="shared" ref="D266:K266" si="181">D$14</f>
+        <f t="shared" ref="D266:K266" si="190">D$14</f>
         <v>45291</v>
       </c>
       <c r="E266" s="224">
-        <f t="shared" si="181"/>
+        <f t="shared" si="190"/>
         <v>45657</v>
       </c>
       <c r="F266" s="224">
-        <f t="shared" si="181"/>
+        <f t="shared" si="190"/>
         <v>46022</v>
       </c>
       <c r="G266" s="224">
-        <f t="shared" si="181"/>
+        <f t="shared" si="190"/>
         <v>46387</v>
       </c>
       <c r="H266" s="224">
-        <f t="shared" si="181"/>
+        <f t="shared" si="190"/>
         <v>46752</v>
       </c>
       <c r="I266" s="224">
-        <f t="shared" si="181"/>
+        <f t="shared" si="190"/>
         <v>47118</v>
       </c>
       <c r="J266" s="224">
-        <f t="shared" si="181"/>
+        <f t="shared" si="190"/>
         <v>47483</v>
       </c>
       <c r="K266" s="224">
-        <f t="shared" si="181"/>
+        <f t="shared" si="190"/>
         <v>47848</v>
       </c>
     </row>
@@ -10928,27 +10928,27 @@
         <v>177494367</v>
       </c>
       <c r="F268" s="183">
-        <f t="shared" ref="F268:K268" si="182">E273</f>
+        <f t="shared" ref="F268:K268" si="191">E273</f>
         <v>172896546</v>
       </c>
       <c r="G268" s="183">
-        <f t="shared" si="182"/>
+        <f t="shared" si="191"/>
         <v>182965452</v>
       </c>
       <c r="H268" s="183">
-        <f t="shared" si="182"/>
+        <f t="shared" si="191"/>
         <v>195235241.11388403</v>
       </c>
       <c r="I268" s="183">
-        <f t="shared" si="182"/>
+        <f t="shared" si="191"/>
         <v>209717874.0450047</v>
       </c>
       <c r="J268" s="183">
-        <f t="shared" si="182"/>
+        <f t="shared" si="191"/>
         <v>226376453.4568519</v>
       </c>
       <c r="K268" s="183">
-        <f t="shared" si="182"/>
+        <f t="shared" si="191"/>
         <v>245036852.63834924</v>
       </c>
     </row>
@@ -10966,23 +10966,23 @@
         <v>43724574</v>
       </c>
       <c r="G269" s="183">
-        <f>G276*G$16</f>
+        <f t="shared" ref="G269:K270" si="192">G276*G$16</f>
         <v>53366787.879486434</v>
       </c>
       <c r="H269" s="183">
-        <f>H276*H$16</f>
+        <f t="shared" si="192"/>
         <v>62991433.055439129</v>
       </c>
       <c r="I269" s="183">
-        <f>I276*I$16</f>
+        <f t="shared" si="192"/>
         <v>72455595.250586137</v>
       </c>
       <c r="J269" s="183">
-        <f>J276*J$16</f>
+        <f t="shared" si="192"/>
         <v>81162402.680470377</v>
       </c>
       <c r="K269" s="183">
-        <f>K276*K$16</f>
+        <f t="shared" si="192"/>
         <v>89288563.051148236</v>
       </c>
     </row>
@@ -11000,23 +11000,23 @@
         <v>27029942</v>
       </c>
       <c r="G270" s="183">
-        <f>G277*G$16</f>
+        <f t="shared" si="192"/>
         <v>32990628.590431124</v>
       </c>
       <c r="H270" s="183">
-        <f>H277*H$16</f>
+        <f t="shared" si="192"/>
         <v>38940454.445260055</v>
       </c>
       <c r="I270" s="183">
-        <f>I277*I$16</f>
+        <f t="shared" si="192"/>
         <v>44791071.885544702</v>
       </c>
       <c r="J270" s="183">
-        <f>J277*J$16</f>
+        <f t="shared" si="192"/>
         <v>50173502.823235251</v>
       </c>
       <c r="K270" s="183">
-        <f>K277*K$16</f>
+        <f t="shared" si="192"/>
         <v>55196985.57922782</v>
       </c>
     </row>
@@ -11068,23 +11068,23 @@
         <v>-58300798</v>
       </c>
       <c r="G272" s="183">
-        <f t="shared" ref="G272:K272" si="183">G279*G$16</f>
+        <f t="shared" ref="G272:K272" si="193">G279*G$16</f>
         <v>-71157384.405181095</v>
       </c>
       <c r="H272" s="183">
-        <f t="shared" si="183"/>
+        <f t="shared" si="193"/>
         <v>-83990545.323453099</v>
       </c>
       <c r="I272" s="183">
-        <f t="shared" si="183"/>
+        <f t="shared" si="193"/>
         <v>-96609723.920333251</v>
       </c>
       <c r="J272" s="183">
-        <f t="shared" si="183"/>
+        <f t="shared" si="193"/>
         <v>-108219072.50299938</v>
       </c>
       <c r="K272" s="183">
-        <f t="shared" si="183"/>
+        <f t="shared" si="193"/>
         <v>-119054206.86672114</v>
       </c>
     </row>
@@ -11109,19 +11109,19 @@
         <v>195235241.11388403</v>
       </c>
       <c r="H273" s="183">
-        <f t="shared" ref="H273:K273" si="184">SUM(H268:H272)</f>
+        <f t="shared" ref="H273:K273" si="194">SUM(H268:H272)</f>
         <v>209717874.0450047</v>
       </c>
       <c r="I273" s="183">
-        <f t="shared" si="184"/>
+        <f t="shared" si="194"/>
         <v>226376453.4568519</v>
       </c>
       <c r="J273" s="183">
-        <f t="shared" si="184"/>
+        <f t="shared" si="194"/>
         <v>245036852.63834924</v>
       </c>
       <c r="K273" s="183">
-        <f t="shared" si="184"/>
+        <f t="shared" si="194"/>
         <v>265565572.51171529</v>
       </c>
     </row>
@@ -11146,19 +11146,19 @@
         <v>0.17317804893570837</v>
       </c>
       <c r="H274" s="334">
-        <f t="shared" ref="H274:K274" si="185">G274</f>
+        <f t="shared" ref="H274:K274" si="195">G274</f>
         <v>0.17317804893570837</v>
       </c>
       <c r="I274" s="334">
-        <f t="shared" si="185"/>
+        <f t="shared" si="195"/>
         <v>0.17317804893570837</v>
       </c>
       <c r="J274" s="334">
-        <f t="shared" si="185"/>
+        <f t="shared" si="195"/>
         <v>0.17317804893570837</v>
       </c>
       <c r="K274" s="334">
-        <f t="shared" si="185"/>
+        <f t="shared" si="195"/>
         <v>0.17317804893570837</v>
       </c>
     </row>
@@ -11177,15 +11177,15 @@
         <v>189</v>
       </c>
       <c r="D276" s="22">
-        <f>D269/D$16</f>
+        <f t="shared" ref="D276:F278" si="196">D269/D$16</f>
         <v>0</v>
       </c>
       <c r="E276" s="22">
-        <f>E269/E$16</f>
+        <f t="shared" si="196"/>
         <v>1.1927602175125E-2</v>
       </c>
       <c r="F276" s="22">
-        <f>F269/F$16</f>
+        <f t="shared" si="196"/>
         <v>1.5194510535745685E-2</v>
       </c>
       <c r="G276" s="209">
@@ -11197,15 +11197,15 @@
         <v>1.5194510535745685E-2</v>
       </c>
       <c r="I276" s="209">
-        <f t="shared" ref="I276:K276" si="186">H276</f>
+        <f t="shared" ref="I276:K276" si="197">H276</f>
         <v>1.5194510535745685E-2</v>
       </c>
       <c r="J276" s="209">
-        <f t="shared" si="186"/>
+        <f t="shared" si="197"/>
         <v>1.5194510535745685E-2</v>
       </c>
       <c r="K276" s="209">
-        <f t="shared" si="186"/>
+        <f t="shared" si="197"/>
         <v>1.5194510535745685E-2</v>
       </c>
     </row>
@@ -11214,15 +11214,15 @@
         <v>190</v>
       </c>
       <c r="D277" s="22">
-        <f>D270/D$16</f>
+        <f t="shared" si="196"/>
         <v>1.3728216801306306E-2</v>
       </c>
       <c r="E277" s="22">
-        <f>E270/E$16</f>
+        <f t="shared" si="196"/>
         <v>9.5905913310619997E-3</v>
       </c>
       <c r="F277" s="22">
-        <f>F270/F$16</f>
+        <f t="shared" si="196"/>
         <v>9.3930415079537376E-3</v>
       </c>
       <c r="G277" s="209">
@@ -11230,19 +11230,19 @@
         <v>9.3930415079537376E-3</v>
       </c>
       <c r="H277" s="209">
-        <f t="shared" ref="H277:K279" si="187">G277</f>
+        <f t="shared" ref="H277:K279" si="198">G277</f>
         <v>9.3930415079537376E-3</v>
       </c>
       <c r="I277" s="209">
-        <f t="shared" si="187"/>
+        <f t="shared" si="198"/>
         <v>9.3930415079537376E-3</v>
       </c>
       <c r="J277" s="209">
-        <f t="shared" si="187"/>
+        <f t="shared" si="198"/>
         <v>9.3930415079537376E-3</v>
       </c>
       <c r="K277" s="209">
-        <f t="shared" si="187"/>
+        <f t="shared" si="198"/>
         <v>9.3930415079537376E-3</v>
       </c>
     </row>
@@ -11251,15 +11251,15 @@
         <v>401</v>
       </c>
       <c r="D278" s="22">
-        <f>D271/D$16</f>
+        <f t="shared" si="196"/>
         <v>0</v>
       </c>
       <c r="E278" s="22">
-        <f>E271/E$16</f>
+        <f t="shared" si="196"/>
         <v>-6.1486832977530263E-4</v>
       </c>
       <c r="F278" s="22">
-        <f>F271/F$16</f>
+        <f t="shared" si="196"/>
         <v>-8.3429430846701145E-4</v>
       </c>
       <c r="G278" s="209">
@@ -11267,19 +11267,19 @@
         <v>-8.3429430846701145E-4</v>
       </c>
       <c r="H278" s="209">
-        <f t="shared" ref="H278" si="188">G278</f>
+        <f t="shared" ref="H278" si="199">G278</f>
         <v>-8.3429430846701145E-4</v>
       </c>
       <c r="I278" s="209">
-        <f t="shared" ref="I278" si="189">H278</f>
+        <f t="shared" ref="I278" si="200">H278</f>
         <v>-8.3429430846701145E-4</v>
       </c>
       <c r="J278" s="209">
-        <f t="shared" ref="J278" si="190">I278</f>
+        <f t="shared" ref="J278" si="201">I278</f>
         <v>-8.3429430846701145E-4</v>
       </c>
       <c r="K278" s="209">
-        <f t="shared" ref="K278" si="191">J278</f>
+        <f t="shared" ref="K278" si="202">J278</f>
         <v>-8.3429430846701145E-4</v>
       </c>
     </row>
@@ -11288,15 +11288,15 @@
         <v>353</v>
       </c>
       <c r="D279" s="22">
-        <f t="shared" ref="D279:F279" si="192">D272/D$16</f>
+        <f t="shared" ref="D279:F279" si="203">D272/D$16</f>
         <v>-3.0174258950275056E-2</v>
       </c>
       <c r="E279" s="22">
-        <f t="shared" si="192"/>
+        <f t="shared" si="203"/>
         <v>-2.3074361877417876E-2</v>
       </c>
       <c r="F279" s="22">
-        <f t="shared" si="192"/>
+        <f t="shared" si="203"/>
         <v>-2.025982207290072E-2</v>
       </c>
       <c r="G279" s="209">
@@ -11304,19 +11304,19 @@
         <v>-2.025982207290072E-2</v>
       </c>
       <c r="H279" s="209">
-        <f t="shared" si="187"/>
+        <f t="shared" si="198"/>
         <v>-2.025982207290072E-2</v>
       </c>
       <c r="I279" s="209">
-        <f t="shared" si="187"/>
+        <f t="shared" si="198"/>
         <v>-2.025982207290072E-2</v>
       </c>
       <c r="J279" s="209">
-        <f t="shared" si="187"/>
+        <f t="shared" si="198"/>
         <v>-2.025982207290072E-2</v>
       </c>
       <c r="K279" s="209">
-        <f t="shared" si="187"/>
+        <f t="shared" si="198"/>
         <v>-2.025982207290072E-2</v>
       </c>
     </row>
@@ -11330,35 +11330,35 @@
         <v>107</v>
       </c>
       <c r="D282" s="48">
-        <f t="shared" ref="D282:K282" si="193">D$13</f>
+        <f t="shared" ref="D282:K282" si="204">D$13</f>
         <v>2023</v>
       </c>
       <c r="E282" s="48">
-        <f t="shared" si="193"/>
+        <f t="shared" si="204"/>
         <v>2024</v>
       </c>
       <c r="F282" s="48">
-        <f t="shared" si="193"/>
+        <f t="shared" si="204"/>
         <v>2025</v>
       </c>
       <c r="G282" s="49">
-        <f t="shared" si="193"/>
+        <f t="shared" si="204"/>
         <v>2026</v>
       </c>
       <c r="H282" s="49">
-        <f t="shared" si="193"/>
+        <f t="shared" si="204"/>
         <v>2027</v>
       </c>
       <c r="I282" s="49">
-        <f t="shared" si="193"/>
+        <f t="shared" si="204"/>
         <v>2028</v>
       </c>
       <c r="J282" s="49">
-        <f t="shared" si="193"/>
+        <f t="shared" si="204"/>
         <v>2029</v>
       </c>
       <c r="K282" s="49">
-        <f t="shared" si="193"/>
+        <f t="shared" si="204"/>
         <v>2030</v>
       </c>
     </row>
@@ -11367,35 +11367,35 @@
         <v>108</v>
       </c>
       <c r="D283" s="335">
-        <f t="shared" ref="D283:K283" si="194">D$14</f>
+        <f t="shared" ref="D283:K283" si="205">D$14</f>
         <v>45291</v>
       </c>
       <c r="E283" s="224">
-        <f t="shared" si="194"/>
+        <f t="shared" si="205"/>
         <v>45657</v>
       </c>
       <c r="F283" s="224">
-        <f t="shared" si="194"/>
+        <f t="shared" si="205"/>
         <v>46022</v>
       </c>
       <c r="G283" s="224">
-        <f t="shared" si="194"/>
+        <f t="shared" si="205"/>
         <v>46387</v>
       </c>
       <c r="H283" s="224">
-        <f t="shared" si="194"/>
+        <f t="shared" si="205"/>
         <v>46752</v>
       </c>
       <c r="I283" s="224">
-        <f t="shared" si="194"/>
+        <f t="shared" si="205"/>
         <v>47118</v>
       </c>
       <c r="J283" s="224">
-        <f t="shared" si="194"/>
+        <f t="shared" si="205"/>
         <v>47483</v>
       </c>
       <c r="K283" s="224">
-        <f t="shared" si="194"/>
+        <f t="shared" si="205"/>
         <v>47848</v>
       </c>
     </row>
@@ -11420,27 +11420,27 @@
         <v>142503563</v>
       </c>
       <c r="F285" s="183">
-        <f t="shared" ref="F285:K285" si="195">E289</f>
+        <f t="shared" ref="F285:K285" si="206">E289</f>
         <v>130756082</v>
       </c>
       <c r="G285" s="183">
-        <f t="shared" si="195"/>
+        <f t="shared" si="206"/>
         <v>136387942</v>
       </c>
       <c r="H285" s="183">
-        <f t="shared" si="195"/>
+        <f t="shared" si="206"/>
         <v>138371018.67622459</v>
       </c>
       <c r="I285" s="183">
-        <f t="shared" si="195"/>
+        <f t="shared" si="206"/>
         <v>140711741.1865674</v>
       </c>
       <c r="J285" s="183">
-        <f t="shared" si="195"/>
+        <f t="shared" si="206"/>
         <v>143404146.08318356</v>
       </c>
       <c r="K285" s="183">
-        <f t="shared" si="195"/>
+        <f t="shared" si="206"/>
         <v>146420090.53360564</v>
       </c>
     </row>
@@ -11618,15 +11618,15 @@
         <v>1.5194510535745685E-2</v>
       </c>
       <c r="I291" s="209">
-        <f t="shared" ref="I291:K292" si="196">H291</f>
+        <f t="shared" ref="I291:K292" si="207">H291</f>
         <v>1.5194510535745685E-2</v>
       </c>
       <c r="J291" s="209">
-        <f t="shared" si="196"/>
+        <f t="shared" si="207"/>
         <v>1.5194510535745685E-2</v>
       </c>
       <c r="K291" s="209">
-        <f t="shared" si="196"/>
+        <f t="shared" si="207"/>
         <v>1.5194510535745685E-2</v>
       </c>
     </row>
@@ -11651,19 +11651,19 @@
         <v>-2.0033305072218234E-3</v>
       </c>
       <c r="H292" s="209">
-        <f t="shared" ref="H292:K292" si="197">G292</f>
+        <f t="shared" ref="H292" si="208">G292</f>
         <v>-2.0033305072218234E-3</v>
       </c>
       <c r="I292" s="209">
-        <f t="shared" si="196"/>
+        <f t="shared" si="207"/>
         <v>-2.0033305072218234E-3</v>
       </c>
       <c r="J292" s="209">
-        <f t="shared" si="196"/>
+        <f t="shared" si="207"/>
         <v>-2.0033305072218234E-3</v>
       </c>
       <c r="K292" s="209">
-        <f t="shared" si="196"/>
+        <f t="shared" si="207"/>
         <v>-2.0033305072218234E-3</v>
       </c>
     </row>
@@ -11692,15 +11692,15 @@
         <v>-1.2626561458672322E-2</v>
       </c>
       <c r="I293" s="209">
-        <f t="shared" ref="I293:K293" si="198">H293</f>
+        <f t="shared" ref="I293:K293" si="209">H293</f>
         <v>-1.2626561458672322E-2</v>
       </c>
       <c r="J293" s="209">
-        <f t="shared" si="198"/>
+        <f t="shared" si="209"/>
         <v>-1.2626561458672322E-2</v>
       </c>
       <c r="K293" s="209">
-        <f t="shared" si="198"/>
+        <f t="shared" si="209"/>
         <v>-1.2626561458672322E-2</v>
       </c>
     </row>
@@ -11714,35 +11714,35 @@
         <v>107</v>
       </c>
       <c r="D296" s="48">
-        <f t="shared" ref="D296:K296" si="199">D$13</f>
+        <f t="shared" ref="D296:K296" si="210">D$13</f>
         <v>2023</v>
       </c>
       <c r="E296" s="48">
-        <f t="shared" si="199"/>
+        <f t="shared" si="210"/>
         <v>2024</v>
       </c>
       <c r="F296" s="48">
-        <f t="shared" si="199"/>
+        <f t="shared" si="210"/>
         <v>2025</v>
       </c>
       <c r="G296" s="49">
-        <f t="shared" si="199"/>
+        <f t="shared" si="210"/>
         <v>2026</v>
       </c>
       <c r="H296" s="49">
-        <f t="shared" si="199"/>
+        <f t="shared" si="210"/>
         <v>2027</v>
       </c>
       <c r="I296" s="49">
-        <f t="shared" si="199"/>
+        <f t="shared" si="210"/>
         <v>2028</v>
       </c>
       <c r="J296" s="49">
-        <f t="shared" si="199"/>
+        <f t="shared" si="210"/>
         <v>2029</v>
       </c>
       <c r="K296" s="49">
-        <f t="shared" si="199"/>
+        <f t="shared" si="210"/>
         <v>2030</v>
       </c>
     </row>
@@ -11751,35 +11751,35 @@
         <v>108</v>
       </c>
       <c r="D297" s="258">
-        <f t="shared" ref="D297:K297" si="200">D$14</f>
+        <f t="shared" ref="D297:K297" si="211">D$14</f>
         <v>45291</v>
       </c>
       <c r="E297" s="224">
-        <f t="shared" si="200"/>
+        <f t="shared" si="211"/>
         <v>45657</v>
       </c>
       <c r="F297" s="224">
-        <f t="shared" si="200"/>
+        <f t="shared" si="211"/>
         <v>46022</v>
       </c>
       <c r="G297" s="224">
-        <f t="shared" si="200"/>
+        <f t="shared" si="211"/>
         <v>46387</v>
       </c>
       <c r="H297" s="224">
-        <f t="shared" si="200"/>
+        <f t="shared" si="211"/>
         <v>46752</v>
       </c>
       <c r="I297" s="224">
-        <f t="shared" si="200"/>
+        <f t="shared" si="211"/>
         <v>47118</v>
       </c>
       <c r="J297" s="224">
-        <f t="shared" si="200"/>
+        <f t="shared" si="211"/>
         <v>47483</v>
       </c>
       <c r="K297" s="224">
-        <f t="shared" si="200"/>
+        <f t="shared" si="211"/>
         <v>47848</v>
       </c>
     </row>
@@ -11793,27 +11793,27 @@
         <v>27899321</v>
       </c>
       <c r="F299" s="183">
-        <f t="shared" ref="F299:K299" si="201">E302</f>
+        <f t="shared" ref="F299:K299" si="212">E302</f>
         <v>21004672</v>
       </c>
       <c r="G299" s="183">
-        <f t="shared" si="201"/>
+        <f t="shared" si="212"/>
         <v>14066392</v>
       </c>
       <c r="H299" s="183">
-        <f t="shared" si="201"/>
+        <f t="shared" si="212"/>
         <v>9066392</v>
       </c>
       <c r="I299" s="183">
-        <f t="shared" si="201"/>
+        <f t="shared" si="212"/>
         <v>6066392</v>
       </c>
       <c r="J299" s="183">
-        <f t="shared" si="201"/>
+        <f t="shared" si="212"/>
         <v>4066392</v>
       </c>
       <c r="K299" s="183">
-        <f t="shared" si="201"/>
+        <f t="shared" si="212"/>
         <v>3066392</v>
       </c>
     </row>
@@ -11896,19 +11896,19 @@
         <v>9066392</v>
       </c>
       <c r="H302" s="183">
-        <f t="shared" ref="H302:K302" si="202">SUM(H299:H301)</f>
+        <f t="shared" ref="H302:K302" si="213">SUM(H299:H301)</f>
         <v>6066392</v>
       </c>
       <c r="I302" s="183">
-        <f t="shared" si="202"/>
+        <f t="shared" si="213"/>
         <v>4066392</v>
       </c>
       <c r="J302" s="183">
-        <f t="shared" si="202"/>
+        <f t="shared" si="213"/>
         <v>3066392</v>
       </c>
       <c r="K302" s="183">
-        <f t="shared" si="202"/>
+        <f t="shared" si="213"/>
         <v>3066392</v>
       </c>
     </row>
@@ -11931,11 +11931,11 @@
         <v>4.3645385931290401E-3</v>
       </c>
       <c r="E304" s="1">
-        <f t="shared" ref="E304:F304" si="203">E300/E$16</f>
+        <f t="shared" ref="E304:F304" si="214">E300/E$16</f>
         <v>1.0092172274202328E-4</v>
       </c>
       <c r="F304" s="1">
-        <f t="shared" si="203"/>
+        <f t="shared" si="214"/>
         <v>0</v>
       </c>
       <c r="G304" s="209">
@@ -11947,15 +11947,15 @@
         <v>0</v>
       </c>
       <c r="I304" s="209">
-        <f t="shared" ref="I304:K304" si="204">H304</f>
+        <f t="shared" ref="I304:K304" si="215">H304</f>
         <v>0</v>
       </c>
       <c r="J304" s="209">
-        <f t="shared" si="204"/>
+        <f t="shared" si="215"/>
         <v>0</v>
       </c>
       <c r="K304" s="209">
-        <f t="shared" si="204"/>
+        <f t="shared" si="215"/>
         <v>0</v>
       </c>
     </row>
@@ -11968,11 +11968,11 @@
         <v>-3.0835535482009496E-3</v>
       </c>
       <c r="E305" s="1">
-        <f t="shared" ref="E305:F305" si="205">E301/E$16</f>
+        <f t="shared" ref="E305:F305" si="216">E301/E$16</f>
         <v>-3.3564934423795508E-3</v>
       </c>
       <c r="F305" s="1">
-        <f t="shared" si="205"/>
+        <f t="shared" si="216"/>
         <v>-2.4110873798325301E-3</v>
       </c>
       <c r="G305" s="209">
@@ -11984,15 +11984,15 @@
         <v>-2.4110873798325301E-3</v>
       </c>
       <c r="I305" s="209">
-        <f t="shared" ref="I305:K305" si="206">H305</f>
+        <f t="shared" ref="I305:K305" si="217">H305</f>
         <v>-2.4110873798325301E-3</v>
       </c>
       <c r="J305" s="209">
-        <f t="shared" si="206"/>
+        <f t="shared" si="217"/>
         <v>-2.4110873798325301E-3</v>
       </c>
       <c r="K305" s="209">
-        <f t="shared" si="206"/>
+        <f t="shared" si="217"/>
         <v>-2.4110873798325301E-3</v>
       </c>
     </row>
@@ -13266,14 +13266,14 @@
       </c>
       <c r="E72" s="357">
         <f ca="1">C72/G72</f>
-        <v>9.6609083296198509E-2</v>
+        <v>9.6498293063060667E-2</v>
       </c>
       <c r="F72" s="71" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="G72" s="359" cm="1">
         <f t="array" aca="1" ref="G72" ca="1">_FV(F72,"Price")</f>
-        <v>52.26</v>
+        <v>52.32</v>
       </c>
     </row>
     <row r="73" spans="2:9" x14ac:dyDescent="0.25">
@@ -13520,7 +13520,7 @@
         <v>0.28516740039140276</v>
       </c>
       <c r="E90" s="120">
-        <f t="dataTable" ref="E90:I94" dt2D="1" dtr="1" r1="C41" r2="H4"/>
+        <f t="dataTable" ref="E90:I94" dt2D="1" dtr="1" r1="C41" r2="H4" ca="1"/>
         <v>4.8452333240374186</v>
       </c>
       <c r="F90" s="120">
@@ -13541,7 +13541,7 @@
         <v>0.28516740039140276</v>
       </c>
       <c r="M90" s="122">
-        <f t="dataTable" ref="M90:Q94" dt2D="1" dtr="1" r1="C41" r2="H4" ca="1"/>
+        <f t="dataTable" ref="M90:Q94" dt2D="1" dtr="1" r1="C41" r2="H4"/>
         <v>5.9044043321622688</v>
       </c>
       <c r="N90" s="122">
@@ -13837,7 +13837,7 @@
         <v>0.28516740039140276</v>
       </c>
       <c r="E99" s="120">
-        <f t="dataTable" ref="E99:I103" dt2D="1" dtr="1" r1="I42" r2="H4"/>
+        <f t="dataTable" ref="E99:I103" dt2D="1" dtr="1" r1="I42" r2="H4" ca="1"/>
         <v>7.5747736378555128</v>
       </c>
       <c r="F99" s="120">
@@ -13858,7 +13858,7 @@
         <v>0.28516740039140276</v>
       </c>
       <c r="M99" s="122">
-        <f t="dataTable" ref="M99:Q103" dt2D="1" dtr="1" r1="I42" r2="H4" ca="1"/>
+        <f t="dataTable" ref="M99:Q103" dt2D="1" dtr="1" r1="I42" r2="H4"/>
         <v>9.1764500952667483</v>
       </c>
       <c r="N99" s="122">

</xml_diff>